<commit_message>
Auto-scrape: doctor in sharjah
</commit_message>
<xml_diff>
--- a/yello_doctor_sharjah.xlsx
+++ b/yello_doctor_sharjah.xlsx
@@ -459,7 +459,11 @@
           <t>'+971 6 565 0690</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/344092/al-abqari-dental-clinic</t>
@@ -482,7 +486,11 @@
           <t>'+971 6 561 7822</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>info@vedhansh.com</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/351899/austin-center-for-rehabilitation-of-person-with-disabilities</t>
@@ -505,7 +513,11 @@
           <t>'+971 6 566 7996</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/354307/sunny-sharqan-medical-centre</t>
@@ -528,7 +540,11 @@
           <t>'+971 6 559 0007</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/352212/al-afdal-medical-center</t>
@@ -551,7 +567,11 @@
           <t>'+971 6 525 3756</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/356351/mulk-physiotherapy-center</t>
@@ -574,7 +594,11 @@
           <t>'+971 6 550 3558</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/343954/ibtisamty-dental-clinic</t>
@@ -597,7 +621,11 @@
           <t>'+971 6 521 8889</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/374124/shifa-al-jazeera-medical-centre-llc</t>
@@ -620,7 +648,11 @@
           <t>'+971 6 506 0000</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17710/zulekha-hospital</t>
@@ -643,7 +675,11 @@
           <t>'+971 6 566 7661</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>alamumahmc@gmail.com</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/352120/dr-uma-maheswari</t>
@@ -666,7 +702,11 @@
           <t>'+971 6 559 1985</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/349515/al-elaj-medical-equipment-tr</t>
@@ -689,7 +729,11 @@
           <t>'+971 6 526 6885</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/347642/art-medical-center</t>
@@ -712,7 +756,11 @@
           <t>'+971 6 568 8600</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/358083/asala-medical-center</t>
@@ -735,7 +783,11 @@
           <t>'+971 6 567 1707</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/347083/al-bawadi-medicaldiagnostic-center</t>
@@ -758,7 +810,11 @@
           <t>'+971 6 555 1575</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/355131/right-medical-centre</t>
@@ -781,7 +837,11 @@
           <t>'+971 6 561 2737</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18028/abrahams-medical-centre</t>
@@ -804,7 +864,11 @@
           <t>'+971 6 530 6161</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/362487/ahlan-medical-center</t>
@@ -827,7 +891,11 @@
           <t>'+971 6 553 0557</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18451/dr-ashok-menon-clinic</t>
@@ -850,7 +918,11 @@
           <t>'+971 6 574 4529</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18042/ahalia-medical-centre</t>
@@ -873,7 +945,11 @@
           <t>'+971 6 535 3582</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342387/al-shams-medicaldiagnostic-centre</t>
@@ -896,7 +972,11 @@
           <t>'+971 6 557 1132</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/207709/bentham-science-publishers-ltd-fzc</t>
@@ -919,7 +999,11 @@
           <t>'+971 6 573 7005</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>info@bissanmc.com</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153264/bissam-medical-centre</t>
@@ -942,7 +1026,11 @@
           <t>'+971 6 522 4422</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/359495/california-dental-clinic</t>
@@ -965,7 +1053,11 @@
           <t>'+971 6 565 2332</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18370/class-medical-centre</t>
@@ -988,7 +1080,11 @@
           <t>'+971 6 575 2200</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18924/prime-medical-center-sharjah</t>
@@ -1011,7 +1107,11 @@
           <t>'+971 6 562 5234</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153395/yathish-kamath-dr-mds-marina-medical-centre</t>
@@ -1034,7 +1134,11 @@
           <t>'+971 6 562 3151</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18032/abubakr-clinic</t>
@@ -1057,7 +1161,11 @@
           <t>'+971 50 424 9032</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/367437/adam-veterinary-medicines-llc</t>
@@ -1080,7 +1188,11 @@
           <t>'+971 6 556 2200</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/222958/al-khaja-medical-clinic</t>
@@ -1103,7 +1215,11 @@
           <t>'+971 6 563 2618</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/361038/al-saha-al-shifa</t>
@@ -1126,7 +1242,11 @@
           <t>'+971 6 575 3888</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17647/bhatia-medical-centre</t>
@@ -1149,7 +1269,11 @@
           <t>'+971 6 563 2100</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18416/doctors-medical-centre</t>
@@ -1172,7 +1296,11 @@
           <t>'+971 52 277 5005</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/364544/dr-zains-homeopathic-clinic-sharjah</t>
@@ -1195,7 +1323,11 @@
           <t>'+971 6 530 9898</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/367702/elite-medical-center</t>
@@ -1218,7 +1350,11 @@
           <t>'+971 6 518 0800</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/362215/ishaq-bin-omran-medical-center-ibo</t>
@@ -1241,7 +1377,11 @@
           <t>'+971 6 525 1000</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/347798/oriana-hospital</t>
@@ -1264,7 +1404,11 @@
           <t>'+971 6 568 2258</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/25748/venniyil-medical-centre</t>
@@ -1287,7 +1431,11 @@
           <t>'+971 6 534 4439</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18143/al-kanary-medical-clinic</t>
@@ -1310,7 +1458,11 @@
           <t>'+971 6 505 7048</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/341538/university-hospital-sharjah</t>
@@ -1333,7 +1485,11 @@
           <t>'+971 600520057</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/371303/hygiene-fresh</t>
@@ -1356,7 +1512,11 @@
           <t>'+971 6 566 7661</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/352098/al-amumah-medical-center</t>
@@ -1379,7 +1539,11 @@
           <t>'+971 6 530 4900</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/353173/lifeway-specialized-medical-centre</t>
@@ -1402,7 +1566,11 @@
           <t>'+971 6 566 8745</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18875/nahar-mampilly-medical-centre</t>
@@ -1425,7 +1593,11 @@
           <t>'+971 6 533 7864</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/148789/unipex-dairy-products-co-ltd</t>
@@ -1448,7 +1620,11 @@
           <t>'+971 6 556 9888</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/350245/al-durrah-radiology-center</t>
@@ -1471,7 +1647,11 @@
           <t>'+971 6 569 1791</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19188/al-watania-veterinary-clinic</t>
@@ -1494,7 +1674,11 @@
           <t>'+971 6 882 2270</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/349667/al-ysra-medical-center</t>
@@ -1517,7 +1701,11 @@
           <t>'+971 6 524 5444</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18380/cosme-surge</t>
@@ -1540,7 +1728,11 @@
           <t>'+971 50 860 6857</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19201/europets-hospital</t>
@@ -1563,7 +1755,11 @@
           <t>'+971 6 534 3803</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/319890/grade-refrigeration-llc</t>
@@ -1586,7 +1782,11 @@
           <t>'+971 6 509 5555</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/371813/gulf-medical-projects</t>
@@ -1609,7 +1809,11 @@
           <t>'+971 6 518 0800</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/360000/ibo</t>
@@ -1632,7 +1836,11 @@
           <t>'+971 6 530 4900</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/366850/lifeway-specialized-medical-centre</t>
@@ -1655,7 +1863,11 @@
           <t>'+971 50 963 8577</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/361312/best-gynaecologist-in-uae</t>
@@ -1678,7 +1890,11 @@
           <t>'+971 6 573 8088</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333177/international-radiology-centre</t>
@@ -1701,7 +1917,11 @@
           <t>'+971 6 525 4446</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/362584/new-hope-ivf</t>
@@ -1724,7 +1944,11 @@
           <t>'+971 6 561 5545</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18070/al-amanah-medical-centre</t>
@@ -1747,7 +1971,11 @@
           <t>'+971 6 561 7277</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18155/al-mahmood-medical-centre</t>
@@ -1770,7 +1998,11 @@
           <t>'+971 6 561 4262</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18224/al-salam-clinic</t>
@@ -1793,7 +2025,11 @@
           <t>'+971 50 252 5966</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/373035/al-sherouq-medical-center</t>
@@ -1816,7 +2052,11 @@
           <t>'+971 6 556 3969</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/373835/al-safwa-radiology-center</t>
@@ -1839,7 +2079,11 @@
           <t>'+971 6 563 6308</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17650/central-private-hospital</t>
@@ -1862,7 +2106,11 @@
           <t>'+971 56 563 6802</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/357446/desert-mart</t>
@@ -1885,7 +2133,11 @@
           <t>'+971 6 555 1666</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18635/emirates-private-poly-clinic</t>
@@ -1908,7 +2160,11 @@
           <t>'+971 6 572 5551</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/365301/eve-fertility-center</t>
@@ -1931,7 +2187,11 @@
           <t>'+971 6 574 4266</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18661/french-rheumatism-clinic</t>
@@ -1954,7 +2214,11 @@
           <t>'+971 50 963 8577</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/363115/gynaecologist-in-sharjah</t>
@@ -1977,7 +2241,11 @@
           <t>'+971 6 539 4466</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/241300/julphar-drug-store-sharjah</t>
@@ -2000,7 +2268,11 @@
           <t>'+971 6 565 2929</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/360495/medical-center-in-sharjah</t>
@@ -2023,7 +2295,11 @@
           <t>'+971 6 574 9610</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18850/minal-medical-clinic</t>
@@ -2046,7 +2322,11 @@
           <t>'+971 6 568 6200</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18880/nathani-medical-centre</t>
@@ -2069,7 +2349,11 @@
           <t>'+971 6 553 6936</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18896/new-medical-centre</t>
@@ -2092,7 +2376,11 @@
           <t>'+971 6 562 5422</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18943/reem-specialists-medical-centre</t>
@@ -2115,7 +2403,11 @@
           <t>'+971 6 558 1515</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E74" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17691/royal-hospital</t>
@@ -2138,7 +2430,11 @@
           <t>'+971 6 575 1222</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17696/sharjah-corniche-hospital</t>
@@ -2161,7 +2457,11 @@
           <t>'+971 6 561 6556</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19000/solanki-dental-center</t>
@@ -2184,7 +2484,11 @@
           <t>'+971 6 530 5882</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18047/ahlan-dental-clinic</t>
@@ -2207,7 +2511,11 @@
           <t>'+971 6 555 1981</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18555/dr-ramzi-assi-dental-clinic</t>
@@ -2230,7 +2538,11 @@
           <t>'+971 6 557 0722</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147645/al-ain-farms-for-livestock-production</t>
@@ -2253,7 +2565,11 @@
           <t>'+971 6 561 3030</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/348714/optimum-medical-center</t>
@@ -2276,7 +2592,11 @@
           <t>'+971 4 323 1889</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/371138/dermahealth</t>
@@ -2295,7 +2615,11 @@
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18770/jwan-murad-fertility-clinic</t>
@@ -2318,7 +2642,11 @@
           <t>'+971 6 556 2727</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152772/abdul-ghani-siddique-ent-clinic-dr</t>
@@ -2341,7 +2669,11 @@
           <t>'+971 6 562 1700</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18057/al-ahalia-regional-medical-centre</t>
@@ -2364,7 +2696,11 @@
           <t>'+971 6 559 9699</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18089/al-buhairah-medical-centre</t>
@@ -2387,7 +2723,11 @@
           <t>'+971 6 559 9147</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19179/al-faseel-veterinarypet-clinic</t>
@@ -2410,7 +2750,11 @@
           <t>'+971 6 562 4456</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18130/al-jahharah-dental-clinic</t>
@@ -2433,7 +2777,11 @@
           <t>'+971 6 561 7577</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18280/alpha-medical-centre</t>
@@ -2456,7 +2804,11 @@
           <t>'+971 6 538 9999</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/228848/al-thiqah-club-for-handicapped</t>
@@ -2479,7 +2831,11 @@
           <t>'+971 6 559 4454</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18296/annie-dental-clinic</t>
@@ -2502,7 +2858,11 @@
           <t>'+971 6 557 3559</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147655/aqsa-international-fzc</t>
@@ -2525,7 +2885,11 @@
           <t>'+971 6 530 3999</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/361501/best-physiotherapy-clinic-in-sharjah</t>
@@ -2548,7 +2912,11 @@
           <t>'+971 6 559 2930</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18388/dablan-dental-clinic</t>
@@ -2571,7 +2939,11 @@
           <t>'+971 6 574 6006</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18437/dr-ali-salem-hindi-clinic</t>
@@ -2594,7 +2966,11 @@
           <t>'+971 6 572 7700</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18449/dr-asad-i-dajani-specialized-centre</t>
@@ -2617,7 +2993,11 @@
           <t>'+971 6 559 1110</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18464/dr-gayatree-medical-centre</t>
@@ -2640,7 +3020,11 @@
           <t>'+971 6 572 7767</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18469/dr-habib-ear-nosethroat-clinic</t>
@@ -2663,7 +3047,11 @@
           <t>'+971 6 563 5029</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18475/dr-hijazis-clinic</t>
@@ -2686,7 +3074,11 @@
           <t>'+971 6 568 5557</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18513/dr-mandar-medical-clinic</t>
@@ -2709,7 +3101,11 @@
           <t>'+971 6 572 1052</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18546/dr-nemat-mossalami</t>
@@ -2732,7 +3128,11 @@
           <t>'+971 6 553 7007</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18575/dr-samir-abou-zeid-clinic</t>
@@ -2755,7 +3155,11 @@
           <t>'+971 6 573 7242</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18590/dr-suha-al-farhan-clinic</t>
@@ -2778,7 +3182,11 @@
           <t>'+971 6 563 9966</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18592/dr-sunny-medical-centre</t>
@@ -2801,7 +3209,11 @@
           <t>'+971 6 562 3844</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18740/ideal-medical-centre</t>
@@ -2824,7 +3236,11 @@
           <t>'+971 6 559 5285</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18746/indulekha-medical-clinic</t>
@@ -2847,7 +3263,11 @@
           <t>'+971 6 524 2688</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18762/jennifer-skin-care-centre</t>
@@ -2870,7 +3290,11 @@
           <t>'+971 6 561 6464</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18810/mampilly-eye-clinic</t>
@@ -2893,7 +3317,11 @@
           <t>'+971 6 569 1400</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18817/marijeh-clinic</t>
@@ -2916,7 +3344,11 @@
           <t>'+971 6 562 5234</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E109" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18819/marina-medical-centre</t>
@@ -2939,7 +3371,11 @@
           <t>'+971 6 563 7719</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E110" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18831/medical-house-for-diagnosistreatment</t>
@@ -2962,7 +3398,11 @@
           <t>'+971 6 562 6922</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18836/medicare-clinic</t>
@@ -2985,7 +3425,11 @@
           <t>'+971 6 539 6200</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E112" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18841/mega-medical-centre</t>
@@ -3008,7 +3452,11 @@
           <t>'+971 6 533 9799</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E113" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18855/modern-dental-clinic</t>
@@ -3031,7 +3479,11 @@
           <t>'+971 6 561 5111</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18954/roy-dental-clinic</t>
@@ -3054,7 +3506,11 @@
           <t>'+971 6 555 3355</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18962/russian-medicalscientific-complex</t>
@@ -3077,7 +3533,11 @@
           <t>'+971 6 556 8888</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E116" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18976/sara-medical-centre</t>
@@ -3100,7 +3560,11 @@
           <t>'+971 6 553 1080</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18986/shamma-dental-clinic</t>
@@ -3123,7 +3587,11 @@
           <t>'+971 6 530 5252</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E118" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342444/sunny-al-nahda-medical-centre</t>
@@ -3146,7 +3614,11 @@
           <t>'+971 55 390 8860</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342445/sunny-speciality-medical-center</t>
@@ -3169,7 +3641,11 @@
           <t>'+971 6 568 2258</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E120" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19049/venniyil-medical-centre</t>
@@ -3192,7 +3668,11 @@
           <t>'+971 6 533 3949</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19070/ziad-e-baghdan-clinic</t>
@@ -3215,7 +3695,11 @@
           <t>'+971 6 530 3999</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/363079/cure-medical-center-physiotherapy</t>
@@ -3238,7 +3722,11 @@
           <t>'+971 6 524 2111</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17673/kuwaiti-hospital</t>
@@ -3261,7 +3749,11 @@
           <t>'+971 55 551 2478</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/369118/yalla-doc</t>
@@ -3284,7 +3776,11 @@
           <t>'+971 6 563 1429</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18173/al-mueed-clinic</t>
@@ -3307,7 +3803,11 @@
           <t>'+971 6 561 9999</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17640/al-zahra-private-hospital</t>
@@ -3326,7 +3826,11 @@
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/317241/cpr-select</t>
@@ -3345,7 +3849,11 @@
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
-      <c r="D128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/368316/niyana</t>
@@ -3368,7 +3876,11 @@
           <t>'+971 6 561 2737</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153514/abrahams-medical-clinic</t>
@@ -3391,7 +3903,11 @@
           <t>'+971 6 886 1202</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr"/>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342379/al-faiez-medical-clinic</t>
@@ -3414,7 +3930,11 @@
           <t>'+971 6 561 7277</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr"/>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152788/al-mahmoud-medical-centre</t>
@@ -3437,7 +3957,11 @@
           <t>'+971 6 542 4255</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr"/>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18237/al-shams-medical-centre</t>
@@ -3460,7 +3984,11 @@
           <t>'+971 6 535 3581</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342388/al-shams-medical-group</t>
@@ -3483,7 +4011,11 @@
           <t>'+971 6 539 7539</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E134" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342395/amritha-medical-centre</t>
@@ -3506,7 +4038,11 @@
           <t>'+971 6 544 4666</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E135" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342396/berlin-medical-centre</t>
@@ -3529,7 +4065,11 @@
           <t>'+971 6 563 9900</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153810/central-pvt-hospital</t>
@@ -3552,7 +4092,11 @@
           <t>'+971 6 577 1822</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E137" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18375/conceive-the-gynaecologyfertility-centre</t>
@@ -3575,7 +4119,11 @@
           <t>'+971 6 533 5555</t>
         </is>
       </c>
-      <c r="D138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E138" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152782/consultants-polymedic</t>
@@ -3598,7 +4146,11 @@
           <t>'+971 6 577 1822</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E139" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153131/conceive</t>
@@ -3621,7 +4173,11 @@
           <t>'+971 55 587 9093</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E140" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/368791/merlin-life-sciences</t>
@@ -3644,7 +4200,11 @@
           <t>'+971 6 574 9610</t>
         </is>
       </c>
-      <c r="D141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E141" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18851/minal-medical-clinic</t>
@@ -3667,7 +4227,11 @@
           <t>'+971 6 882 8486</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E142" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153426/new-zulekha-medical-centre</t>
@@ -3690,7 +4254,11 @@
           <t>'+971 6 558 3351</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18948/riaz-medical-center</t>
@@ -3713,7 +4281,11 @@
           <t>'+971 6 575 0077</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18964/saba-physiotherapy-center</t>
@@ -3736,7 +4308,11 @@
           <t>'+971 6 556 9900</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr"/>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E145" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153829/saudi-german-hospital-group</t>
@@ -3759,7 +4335,11 @@
           <t>'+971 6 573 7888</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E146" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18982/scottish-dental-clinic</t>
@@ -3782,7 +4362,11 @@
           <t>'+971 6 538 8966</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153091/sunnys-clinic-dr</t>
@@ -3805,7 +4389,11 @@
           <t>'+971 6 566 2416</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E148" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/148778/universal-mediators-fze</t>
@@ -3828,7 +4416,11 @@
           <t>'+971 6 574 4734</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E149" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19059/widex-emirates-hearing-care</t>
@@ -3851,7 +4443,11 @@
           <t>'+971 6 553 8156</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E150" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19073/zulekha-medical-centre</t>
@@ -3874,7 +4470,11 @@
           <t>'+971 6 538 6444</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E151" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342367/al-qassimi-hospital</t>
@@ -3897,7 +4497,11 @@
           <t>'+971 6 538 6444</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E152" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153819/al-qasimia-hospital</t>
@@ -3920,7 +4524,11 @@
           <t>'+971 6 511 9000</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342439/private-rehabilitation-center</t>
@@ -3943,7 +4551,11 @@
           <t>'+971 6 566 0008</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr"/>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E154" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333696/dr-anwar-pasha-medical-clinic</t>
@@ -3966,7 +4578,11 @@
           <t>'+971 6 562 3151</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E155" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153754/abubakar-clinic</t>
@@ -3989,7 +4605,11 @@
           <t>'+971 6 574 0091</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18038/afif-medical-centre</t>
@@ -4012,7 +4632,11 @@
           <t>'+971 6 574 2333</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr"/>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E157" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152785/ahmed-bishr-medical-centre-dr</t>
@@ -4035,7 +4659,11 @@
           <t>'+971 6 556 8777</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E158" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18074/al-amoodi-medical-center</t>
@@ -4058,7 +4686,11 @@
           <t>'+971 6 556 8777</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr"/>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153495/al-amoodi-medical-centre</t>
@@ -4081,7 +4713,11 @@
           <t>'+971 6 533 1551</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr"/>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E160" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147633/al-buheira-lacnor-dairies-co-ltd</t>
@@ -4104,7 +4740,11 @@
           <t>'+971 6 533 1894</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr"/>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E161" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/148779/al-fatha-fstuff-trading-co</t>
@@ -4127,7 +4767,11 @@
           <t>'+971 6 561 8825</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr"/>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E162" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18277/alia-clinic</t>
@@ -4150,7 +4794,11 @@
           <t>'+971 6 574 6006</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr"/>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E163" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153752/ali-salem-hindi-clinic-dr</t>
@@ -4173,7 +4821,11 @@
           <t>'+971 6 556 2200</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr"/>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18146/al-khajah-medical-group</t>
@@ -4196,7 +4848,11 @@
           <t>'+971 6 564 6252</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr"/>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E165" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153349/al-lulu-medical-centre</t>
@@ -4219,7 +4875,11 @@
           <t>'+971 6 543 3772</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr"/>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/148774/al-maydan-refrigeration</t>
@@ -4242,7 +4902,11 @@
           <t>'+971 6 882 3334</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr"/>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153757/al-maliha-medical-centre</t>
@@ -4265,7 +4929,11 @@
           <t>'+971 6 556 1610</t>
         </is>
       </c>
-      <c r="D168" t="inlineStr"/>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18188/al-nawa-medical-centre</t>
@@ -4288,7 +4956,11 @@
           <t>'+971 6 531 5152</t>
         </is>
       </c>
-      <c r="D169" t="inlineStr"/>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153376/al-nahdah-medical-centre</t>
@@ -4311,7 +4983,11 @@
           <t>'+971 6 573 1735</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr"/>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18230/al-saraj-medical-centre</t>
@@ -4334,7 +5010,11 @@
           <t>'+971 6 553 8787</t>
         </is>
       </c>
-      <c r="D171" t="inlineStr"/>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E171" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18231/al-sarraf-medical-center</t>
@@ -4357,7 +5037,11 @@
           <t>'+971 6 561 7413</t>
         </is>
       </c>
-      <c r="D172" t="inlineStr"/>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18233/al-sawami-medical-clinic</t>
@@ -4380,7 +5064,11 @@
           <t>'+971 6 543 2898</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr"/>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E173" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153390/al-safeer-medical-centre</t>
@@ -4403,7 +5091,11 @@
           <t>'+971 6 555 8441</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr"/>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E174" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18252/al-taif-medical-centre</t>
@@ -4426,7 +5118,11 @@
           <t>'+971 6 559 9011</t>
         </is>
       </c>
-      <c r="D175" t="inlineStr"/>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18262/al-wahda-dental-clinic</t>
@@ -4449,7 +5145,11 @@
           <t>'+971 6 534 6767</t>
         </is>
       </c>
-      <c r="D176" t="inlineStr"/>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E176" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147646/arla-nfpc</t>
@@ -4472,7 +5172,11 @@
           <t>'+971 6 553 0557</t>
         </is>
       </c>
-      <c r="D177" t="inlineStr"/>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E177" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153292/ashok-menon-clinic-dr</t>
@@ -4495,7 +5199,11 @@
           <t>'+971 6 561 5434</t>
         </is>
       </c>
-      <c r="D178" t="inlineStr"/>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E178" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153508/ayurvedic-herbal-health-centre</t>
@@ -4518,7 +5226,11 @@
           <t>'+971 6 534 1334</t>
         </is>
       </c>
-      <c r="D179" t="inlineStr"/>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E179" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/148783/baras-al-khaimahat-international</t>
@@ -4541,7 +5253,11 @@
           <t>'+971 6 574 6646</t>
         </is>
       </c>
-      <c r="D180" t="inlineStr"/>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E180" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18329/basil-medical-clinic</t>
@@ -4564,7 +5280,11 @@
           <t>'+971 6 562 7778</t>
         </is>
       </c>
-      <c r="D181" t="inlineStr"/>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E181" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342399/dallas-medical-center</t>
@@ -4587,7 +5307,11 @@
           <t>'+971 6 572 7515</t>
         </is>
       </c>
-      <c r="D182" t="inlineStr"/>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E182" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18401/dental-care-centre</t>
@@ -4610,7 +5334,11 @@
           <t>'+971 6 572 7044</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr"/>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E183" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153375/dhia-h-mahdi-dr</t>
@@ -4633,7 +5361,11 @@
           <t>'+971 6 562 1777</t>
         </is>
       </c>
-      <c r="D184" t="inlineStr"/>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E184" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18411/diana-dental-clinic</t>
@@ -4656,7 +5388,11 @@
           <t>'+971 6 574 2333</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr"/>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E185" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18431/dr-ahmed-bishr-medical-centre</t>
@@ -4679,7 +5415,11 @@
           <t>'+971 6 523 8883</t>
         </is>
       </c>
-      <c r="D186" t="inlineStr"/>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E186" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342400/dr-amal-al-qedrah-specialist-clinic</t>
@@ -4702,7 +5442,11 @@
           <t>'+971 6 555 1937</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr"/>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E187" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18491/dr-joseph-dental-clinic</t>
@@ -4725,7 +5469,11 @@
           <t>'+971 6 563 6192</t>
         </is>
       </c>
-      <c r="D188" t="inlineStr"/>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E188" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18530/dr-mohd-tharwat-dental-clinic</t>
@@ -4748,7 +5496,11 @@
           <t>'+971 6 562 6525</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr"/>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E189" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18578/dr-sanjay-medical-centre</t>
@@ -4771,7 +5523,11 @@
           <t>'+971 6 533 8732</t>
         </is>
       </c>
-      <c r="D190" t="inlineStr"/>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E190" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18567/dr-sadeq-al-sahaf</t>
@@ -4794,7 +5550,11 @@
           <t>'+971 6 574 2434</t>
         </is>
       </c>
-      <c r="D191" t="inlineStr"/>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E191" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18576/dr-samir-ali-murad-dental-clinic</t>
@@ -4817,7 +5577,11 @@
           <t>'+971 9 238 6389</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr"/>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E192" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153118/east-coast-clinic</t>
@@ -4840,7 +5604,11 @@
           <t>'+971 6 556 3433</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr"/>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153344/enjab-medical-centre</t>
@@ -4863,7 +5631,11 @@
           <t>'+971 6 562 3722</t>
         </is>
       </c>
-      <c r="D194" t="inlineStr"/>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E194" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18636/esfandyar-polyclinic</t>
@@ -4886,7 +5658,11 @@
           <t>'+971 6 577 5700</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr"/>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E195" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153364/fetal-medicine-clinic</t>
@@ -4909,7 +5685,11 @@
           <t>'+971 6 553 5228</t>
         </is>
       </c>
-      <c r="D196" t="inlineStr"/>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E196" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18666/future-orthodontic-dental-clinic</t>
@@ -4932,7 +5712,11 @@
           <t>'+971 6 575 0280</t>
         </is>
       </c>
-      <c r="D197" t="inlineStr"/>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E197" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18679/german-medical-clinic</t>
@@ -4955,7 +5739,11 @@
           <t>'+971 6 542 3399</t>
         </is>
       </c>
-      <c r="D198" t="inlineStr"/>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E198" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18690/gopi-medical-clinic</t>
@@ -4978,7 +5766,11 @@
           <t>'+971 6 561 6016</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr"/>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E199" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18695/gulf-ayurvedic-centre</t>
@@ -5001,7 +5793,11 @@
           <t>'+971 2 621 7715</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr"/>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E200" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/239069/gulf-medical-projects-company</t>
@@ -5024,7 +5820,11 @@
           <t>'+971 6 572 7767</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr"/>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E201" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153532/habib-dr-ent-clinic</t>
@@ -5047,7 +5847,11 @@
           <t>'+971 6 559 9234</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr"/>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E202" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18709/hakim-medical-center</t>
@@ -5070,7 +5874,11 @@
           <t>'+971 6 562 5634</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr"/>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E203" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18758/jeena-clinic</t>
@@ -5093,7 +5901,11 @@
           <t>'+971 6 555 1937</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr"/>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E204" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153244/joseph-dental-clinic-dr</t>
@@ -5116,7 +5928,11 @@
           <t>'+971 9 277 7002</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr"/>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E205" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153294/kalba-medical-center</t>
@@ -5139,7 +5955,11 @@
           <t>'+971 6 561 8335</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr"/>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E206" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18779/khalid-polyclinic</t>
@@ -5162,7 +5982,11 @@
           <t>'+971 6 559 9828</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr"/>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E207" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18788/knan-dental-clinic</t>
@@ -5185,7 +6009,11 @@
           <t>'+971 6 543 7388</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr"/>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E208" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147640/kuwait-danish-dairy-co-kcsc-the</t>
@@ -5208,7 +6036,11 @@
           <t>'+971 6 563 0447</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr"/>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E209" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153362/laika-wali-medical-clinic</t>
@@ -5231,7 +6063,11 @@
           <t>'+971 6 533 3951</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr"/>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E210" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153360/legend-clinic</t>
@@ -5254,7 +6090,11 @@
           <t>'+971 6 561 6464</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr"/>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E211" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153527/mampilly-clinic</t>
@@ -5277,7 +6117,11 @@
           <t>'+971 6 568 5557</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr"/>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E212" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153423/mandar-medical-clinic-dr</t>
@@ -5300,7 +6144,11 @@
           <t>'+971 6 544 0555</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr"/>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E213" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/243414/med-pharma</t>
@@ -5323,7 +6171,11 @@
           <t>'+971 6 572 2999</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr"/>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E214" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153332/metawi-medical-paediatrician-clinic</t>
@@ -5346,7 +6198,11 @@
           <t>'+971 6 556 5656</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr"/>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E215" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153384/mohd-a-el-nounou-clinic-dr</t>
@@ -5369,7 +6225,11 @@
           <t>'+971 6 563 6192</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr"/>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E216" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153730/mohd-tharwat-dental-clinic-dr</t>
@@ -5392,7 +6252,11 @@
           <t>'+971 6 553 8238</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr"/>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E217" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153506/mouen-junblat-medical-centre-dr</t>
@@ -5415,7 +6279,11 @@
           <t>'+971 6 573 6500</t>
         </is>
       </c>
-      <c r="D218" t="inlineStr"/>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E218" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147666/national-agric-dev-co-the</t>
@@ -5438,7 +6306,11 @@
           <t>'+971 6 562 3834</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr"/>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E219" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153394/nathani-clinic</t>
@@ -5461,7 +6333,11 @@
           <t>'+971 6 523 3300</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E220" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/342435/national-center-for-modern-medicine</t>
@@ -5484,7 +6360,11 @@
           <t>'+971 6 568 4974</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr"/>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E221" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18905/noor-clinic</t>
@@ -5507,7 +6387,11 @@
           <t>'+971 6 573 7735</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr"/>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E222" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18911/our-own-medical-and-diagnostics-center</t>
@@ -5530,7 +6414,11 @@
           <t>'+971 6 573 7735</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr"/>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E223" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153243/our-own-medicaldiagnostics-center</t>
@@ -5553,7 +6441,11 @@
           <t>'+971 6 557 1797</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr"/>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E224" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/246461/pharmacare-limited</t>
@@ -5576,7 +6468,11 @@
           <t>'+971 6 562 5890</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr"/>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E225" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18928/private-eye-clinic</t>
@@ -5599,7 +6495,11 @@
           <t>'+971 6 573 7789</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr"/>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E226" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153370/psychiatric-clinic</t>
@@ -5622,7 +6522,11 @@
           <t>'+971 6 574 4677</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr"/>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E227" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153366/raad-al-qasik-medical-centre-dr</t>
@@ -5645,7 +6549,11 @@
           <t>'+971 6 572 2330</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr"/>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E228" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153348/rania-al-qedrah-specialized-clinic-dr</t>
@@ -5668,7 +6576,11 @@
           <t>'+971 6 562 0831</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr"/>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153379/reem-medical-diagnostic-centre</t>
@@ -5691,7 +6603,11 @@
           <t>'+971 6 562 5422</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr"/>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E230" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153729/reem-specialists-medical-center</t>
@@ -5714,7 +6630,11 @@
           <t>'+971 6 561 2900</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr"/>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18950/rishil-poly-clinic</t>
@@ -5737,7 +6657,11 @@
           <t>'+971 6 533 8732</t>
         </is>
       </c>
-      <c r="D232" t="inlineStr"/>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E232" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153324/sadeq-al-sahaf-dr</t>
@@ -5760,7 +6684,11 @@
           <t>'+971 6 567 6027</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr"/>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E233" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18969/sajida-medical-centre</t>
@@ -5783,7 +6711,11 @@
           <t>'+971 6 553 7007</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E234" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153248/samir-abu-zied-clinic-dr</t>
@@ -5806,7 +6738,11 @@
           <t>'+971 6 556 5589</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E235" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153357/samia-khedr-medical-clinic-dr</t>
@@ -5829,7 +6765,11 @@
           <t>'+971 6 574 2434</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr"/>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E236" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153760/samir-ali-murad-dental-clinic-dr</t>
@@ -5852,7 +6792,11 @@
           <t>'+971 6 562 6525</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr"/>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E237" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153257/sanjay-medical-centre-dr</t>
@@ -5875,7 +6819,11 @@
           <t>'+971 6 568 2670</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr"/>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E238" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18977/sarhad-medical-clinic</t>
@@ -5898,7 +6846,11 @@
           <t>'+971 6 562 6957</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr"/>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E239" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18978/sasils-dental-clinic</t>
@@ -5921,7 +6873,11 @@
           <t>'+971 6 563 6308</t>
         </is>
       </c>
-      <c r="D240" t="inlineStr"/>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E240" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153824/shakir-s-vali-dr</t>
@@ -5944,7 +6900,11 @@
           <t>'+971 6 561 6556</t>
         </is>
       </c>
-      <c r="D241" t="inlineStr"/>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E241" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153335/solanki-dental-centre</t>
@@ -5967,7 +6927,11 @@
           <t>'+971 6 573 7242</t>
         </is>
       </c>
-      <c r="D242" t="inlineStr"/>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E242" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153356/suha-al-farhan-children-dentist-dr</t>
@@ -5990,7 +6954,11 @@
           <t>'+971 6 573 0666</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr"/>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E243" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19012/swedish-clinic</t>
@@ -6013,7 +6981,11 @@
           <t>'+971 6 533 9196</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr"/>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E244" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/147639/united-dairies</t>
@@ -6036,7 +7008,11 @@
           <t>'+971 6 568 2258</t>
         </is>
       </c>
-      <c r="D245" t="inlineStr"/>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E245" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153114/venniyil-clinic</t>
@@ -6059,7 +7035,11 @@
           <t>'+971 6 572 1313</t>
         </is>
       </c>
-      <c r="D246" t="inlineStr"/>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E246" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153351/wassim-kabbani-clinic-dr</t>
@@ -6082,7 +7062,11 @@
           <t>'+971 6 577 1757</t>
         </is>
       </c>
-      <c r="D247" t="inlineStr"/>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E247" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153820/wilson-specialized-hospital</t>
@@ -6105,7 +7089,11 @@
           <t>'+971 6 577 1757</t>
         </is>
       </c>
-      <c r="D248" t="inlineStr"/>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E248" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19052/w-wilson-health-care-group</t>
@@ -6128,7 +7116,11 @@
           <t>'+971 6 538 8205</t>
         </is>
       </c>
-      <c r="D249" t="inlineStr"/>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E249" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18159/al-maliky-dental-clinic</t>
@@ -6147,7 +7139,11 @@
         </is>
       </c>
       <c r="C250" t="inlineStr"/>
-      <c r="D250" t="inlineStr"/>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E250" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/226714/al-riyadh-medical-equipments-centre</t>
@@ -6170,7 +7166,11 @@
           <t>'+971 6 568 5022</t>
         </is>
       </c>
-      <c r="D251" t="inlineStr"/>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E251" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18246/al-shrook-polyclinic</t>
@@ -6189,7 +7189,11 @@
         </is>
       </c>
       <c r="C252" t="inlineStr"/>
-      <c r="D252" t="inlineStr"/>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E252" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/228491/al-taheal-medical-equipment</t>
@@ -6212,7 +7216,11 @@
           <t>'+971 6 568 7728</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr"/>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E253" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18284/ambegaokar-clinic</t>
@@ -6235,7 +7243,11 @@
           <t>'+971 6 562 0404</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr"/>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E254" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18397/delta-medical-clinic</t>
@@ -6258,7 +7270,11 @@
           <t>'+971 6 573 6466</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr"/>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E255" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18501/dr-labib-al-hasan-medical-clinic</t>
@@ -6281,7 +7297,11 @@
           <t>'+971 6 561 5754</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr"/>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E256" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18730/hyma-medical-clinic</t>
@@ -6304,7 +7324,11 @@
           <t>'+971 6 561 5754</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr"/>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E257" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153325/hyma-medical-clinic-hemalatha-dr</t>
@@ -6323,7 +7347,11 @@
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
-      <c r="D258" t="inlineStr"/>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E258" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/240124/ibn-rushd-medical-drugs-equipment-store</t>
@@ -6346,7 +7374,11 @@
           <t>'+971 6 573 6466</t>
         </is>
       </c>
-      <c r="D259" t="inlineStr"/>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E259" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153434/labib-al-hasan-medical-clinic-dr</t>
@@ -6369,7 +7401,11 @@
           <t>'+971 6 563 4347</t>
         </is>
       </c>
-      <c r="D260" t="inlineStr"/>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E260" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18839/mediplus-diagnostic-centre</t>
@@ -6392,7 +7428,11 @@
           <t>'+971 9 277 7351</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr"/>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E261" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153411/zafar-dental-clinic</t>
@@ -6415,7 +7455,11 @@
           <t>'+971 6 561 4266</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr"/>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E262" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18091/al-dallah-medical-clinic</t>
@@ -6438,7 +7482,11 @@
           <t>'+971 6 555 1231</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr"/>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E263" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18136/al-jawhara-medical-center</t>
@@ -6461,7 +7509,11 @@
           <t>'+971 6 564 6252</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr"/>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E264" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18150/al-lulu-medical-center</t>
@@ -6484,7 +7536,11 @@
           <t>'+971 6 568 6511</t>
         </is>
       </c>
-      <c r="D265" t="inlineStr"/>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E265" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18179/al-mushtaq-medical-centre</t>
@@ -6507,7 +7563,11 @@
           <t>'+971 6 538 6444</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr"/>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E266" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/17633/al-qassemi-hospital</t>
@@ -6530,7 +7590,11 @@
           <t>'+971 6 568 7893</t>
         </is>
       </c>
-      <c r="D267" t="inlineStr"/>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E267" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18209/al-rai-medical-centre</t>
@@ -6553,7 +7617,11 @@
           <t>'+971 6 561 9999</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr"/>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E268" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153809/al-zahra-pvt-hospital</t>
@@ -6576,7 +7644,11 @@
           <t>'+971 6 568 1717</t>
         </is>
       </c>
-      <c r="D269" t="inlineStr"/>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E269" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18333/bhatia-clinic</t>
@@ -6599,7 +7671,11 @@
           <t>'+971 6 563 6552</t>
         </is>
       </c>
-      <c r="D270" t="inlineStr"/>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E270" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18387/dabbous-medical-centre</t>
@@ -6622,7 +7698,11 @@
           <t>'+971 6 572 5626</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr"/>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E271" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18392/davis-dental-clinic</t>
@@ -6645,7 +7725,11 @@
           <t>'+971 6 553 8238</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E272" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18532/dr-mouen-junblat-dental-clinic</t>
@@ -6668,7 +7752,11 @@
           <t>'+971 6 574 1313</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr"/>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18550/dr-oras-sharif-clinic</t>
@@ -6691,7 +7779,11 @@
           <t>'+971 6 572 1919</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr"/>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E274" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18570/dr-said-h-muwafi</t>
@@ -6714,7 +7806,11 @@
           <t>'+971 6 572 2458</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr"/>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E275" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18572/dr-saleh-mohammed-saleh</t>
@@ -6733,7 +7829,11 @@
         </is>
       </c>
       <c r="C276" t="inlineStr"/>
-      <c r="D276" t="inlineStr"/>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E276" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/236155/dynamic-rehab-medical-centre</t>
@@ -6756,7 +7856,11 @@
           <t>'+971 6 555 2150</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr"/>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E277" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18650/family-clinic</t>
@@ -6779,7 +7883,11 @@
           <t>'+971 6 561 8300</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr"/>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E278" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18763/jessy-clinic</t>
@@ -6802,7 +7910,11 @@
           <t>'+971 6 561 5307</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr"/>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E279" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18798/lyla-dental-clinic</t>
@@ -6825,7 +7937,11 @@
           <t>'+971 6 568 3405</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr"/>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E280" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18951/rolla-clinic</t>
@@ -6848,7 +7964,11 @@
           <t>'+971 6 563 5201</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr"/>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E281" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18952/romira-paediatric-clinic</t>
@@ -6871,7 +7991,11 @@
           <t>'+971 6 573 6800</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr"/>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E282" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/19006/specialized-medical-center</t>
@@ -6894,7 +8018,11 @@
           <t>'+971 6 572 4484</t>
         </is>
       </c>
-      <c r="D283" t="inlineStr"/>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E283" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18468/dr-gills-clinic</t>
@@ -6913,7 +8041,11 @@
         </is>
       </c>
       <c r="C284" t="inlineStr"/>
-      <c r="D284" t="inlineStr"/>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E284" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/218254/al-ameen-medical-centre</t>
@@ -6936,7 +8068,11 @@
           <t>'+971 6 555 1981</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr"/>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E285" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152776/assi-dental-clinic-dr</t>
@@ -6959,7 +8095,11 @@
           <t>'+971 6 538 6444</t>
         </is>
       </c>
-      <c r="D286" t="inlineStr"/>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E286" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153808/new-al-qassemiya-hospital</t>
@@ -6982,7 +8122,11 @@
           <t>'+971 6 542 0066</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr"/>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E287" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/364526/modern-clinic</t>
@@ -7005,7 +8149,11 @@
           <t>'+971 6 573 3440</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr"/>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E288" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153339/abdulla-semrin-clinic-dr</t>
@@ -7028,7 +8176,11 @@
           <t>'+971 6 555 1231</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr"/>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E289" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153504/adnan-ballout-clinic-dr</t>
@@ -7051,7 +8203,11 @@
           <t>'+971 6 556 1220</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr"/>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E290" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18036/advanced-eye-clinic</t>
@@ -7074,7 +8230,11 @@
           <t>'+971 6 562 1700</t>
         </is>
       </c>
-      <c r="D291" t="inlineStr"/>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E291" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18059/al-ahlia-regional-medical-centre</t>
@@ -7097,7 +8257,11 @@
           <t>'+971 6 561 5545</t>
         </is>
       </c>
-      <c r="D292" t="inlineStr"/>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E292" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18071/al-amanah-medical-centre</t>
@@ -7120,7 +8284,11 @@
           <t>'+971 6 561 6828</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr"/>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E293" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152760/al-ansari-clinic</t>
@@ -7143,7 +8311,11 @@
           <t>'+971 6 534 8384</t>
         </is>
       </c>
-      <c r="D294" t="inlineStr"/>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E294" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/302790/al-araimi-gen-trading-llc</t>
@@ -7166,7 +8338,11 @@
           <t>'+971 6 555 9905</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr"/>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E295" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333726/al-alfiah-dental-clinic</t>
@@ -7189,7 +8365,11 @@
           <t>'+971 6 543 1763</t>
         </is>
       </c>
-      <c r="D296" t="inlineStr"/>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E296" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18085/al-barakah-medical-clinic</t>
@@ -7212,7 +8392,11 @@
           <t>'+971 6 543 1763</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr"/>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E297" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152771/al-baras-al-khaimahah-medical-clinic</t>
@@ -7235,7 +8419,11 @@
           <t>'+971 6 572 7175</t>
         </is>
       </c>
-      <c r="D298" t="inlineStr"/>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E298" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153105/al-batool-complex-medical</t>
@@ -7258,7 +8446,11 @@
           <t>'+971 6 533 6176</t>
         </is>
       </c>
-      <c r="D299" t="inlineStr"/>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E299" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18095/al-darary-medical-centre</t>
@@ -7281,7 +8473,11 @@
           <t>'+971 6 532 0800</t>
         </is>
       </c>
-      <c r="D300" t="inlineStr"/>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E300" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153731/al-diyafah-medical-centre</t>
@@ -7304,7 +8500,11 @@
           <t>'+971 6 534 3870</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr"/>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E301" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/331951/al-fanar-food-industries-llc</t>
@@ -7327,7 +8527,11 @@
           <t>'+971 6 556 2444</t>
         </is>
       </c>
-      <c r="D302" t="inlineStr"/>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E302" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152778/al-huda-polyclinic</t>
@@ -7350,7 +8554,11 @@
           <t>'+971 6 561 3613</t>
         </is>
       </c>
-      <c r="D303" t="inlineStr"/>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E303" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18128/al-ishraf-medical-centre</t>
@@ -7373,7 +8581,11 @@
           <t>'+971 6 561 3613</t>
         </is>
       </c>
-      <c r="D304" t="inlineStr"/>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E304" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153305/al-ishraf-medical-center</t>
@@ -7396,7 +8608,11 @@
           <t>'+971 6 556 5660</t>
         </is>
       </c>
-      <c r="D305" t="inlineStr"/>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E305" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18156/al-majaz-medical-centre</t>
@@ -7419,7 +8635,11 @@
           <t>'+971 6 573 9545</t>
         </is>
       </c>
-      <c r="D306" t="inlineStr"/>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E306" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18176/al-muntasir-medical-centre</t>
@@ -7442,7 +8662,11 @@
           <t>'+971 6 538 8205</t>
         </is>
       </c>
-      <c r="D307" t="inlineStr"/>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E307" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18160/al-maliky-dental-clinic</t>
@@ -7465,7 +8689,11 @@
           <t>'+971 4 338 3339</t>
         </is>
       </c>
-      <c r="D308" t="inlineStr"/>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E308" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/224696/al-mufid-trading-company-llc</t>
@@ -7488,7 +8716,11 @@
           <t>'+971 6 561 8899</t>
         </is>
       </c>
-      <c r="D309" t="inlineStr"/>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E309" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18185/al-nakheel-medical-centre</t>
@@ -7511,7 +8743,11 @@
           <t>'+971 6 561 2696</t>
         </is>
       </c>
-      <c r="D310" t="inlineStr"/>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E310" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18181/al-naeem-medical-center</t>
@@ -7534,7 +8770,11 @@
           <t>'+971 6 533 4415</t>
         </is>
       </c>
-      <c r="D311" t="inlineStr"/>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E311" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18204/al-raha-medical-center</t>
@@ -7557,7 +8797,11 @@
           <t>'+971 6 533 3913</t>
         </is>
       </c>
-      <c r="D312" t="inlineStr"/>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E312" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/318786/al-rubiyan-trading-company-llc</t>
@@ -7580,7 +8824,11 @@
           <t>'+971 6 557 5075</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr"/>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E313" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/332063/al-rimal-foodstuff-inds-fzc</t>
@@ -7603,7 +8851,11 @@
           <t>'+971 6 562 3949</t>
         </is>
       </c>
-      <c r="D314" t="inlineStr"/>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E314" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18218/al-saadah-medical-center</t>
@@ -7626,7 +8878,11 @@
           <t>'+971 6 563 5211</t>
         </is>
       </c>
-      <c r="D315" t="inlineStr"/>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E315" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18219/al-safa-clinic</t>
@@ -7649,7 +8905,11 @@
           <t>'+971 6 563 2618</t>
         </is>
       </c>
-      <c r="D316" t="inlineStr"/>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E316" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18223/al-saha-wa-al-shifaa-specialities-complex</t>
@@ -7672,7 +8932,11 @@
           <t>'+971 6 532 5327</t>
         </is>
       </c>
-      <c r="D317" t="inlineStr"/>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E317" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/148788/al-shams-food-industries</t>
@@ -7695,7 +8959,11 @@
           <t>'+971(6)379735</t>
         </is>
       </c>
-      <c r="D318" t="inlineStr"/>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E318" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/299592/al-shulla-vet-center</t>
@@ -7718,7 +8986,11 @@
           <t>'+971 6 563 2618</t>
         </is>
       </c>
-      <c r="D319" t="inlineStr"/>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E319" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333639/al-soha-and-al-shifa-specialities-complex</t>
@@ -7741,7 +9013,11 @@
           <t>'+971 6 572 7757</t>
         </is>
       </c>
-      <c r="D320" t="inlineStr"/>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E320" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153338/al-thequah-clinic</t>
@@ -7764,7 +9040,11 @@
           <t>'+971 6 534 7494</t>
         </is>
       </c>
-      <c r="D321" t="inlineStr"/>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E321" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18259/al-wafir-medical-centre</t>
@@ -7787,7 +9067,11 @@
           <t>'+971 6 574 9666</t>
         </is>
       </c>
-      <c r="D322" t="inlineStr"/>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E322" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18266/al-widad-specialist-clinic</t>
@@ -7810,7 +9094,11 @@
           <t>'+971 6 574 9666</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr"/>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E323" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333683/al-widad-specialist</t>
@@ -7833,7 +9121,11 @@
           <t>'+971 6 561 9999</t>
         </is>
       </c>
-      <c r="D324" t="inlineStr"/>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E324" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/299495/al-zahar-hospital</t>
@@ -7856,7 +9148,11 @@
           <t>'+971 6 556 5564</t>
         </is>
       </c>
-      <c r="D325" t="inlineStr"/>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E325" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18282/amal-abdel-kader-dental-clinic</t>
@@ -7879,7 +9175,11 @@
           <t>'+971 6 563 0555</t>
         </is>
       </c>
-      <c r="D326" t="inlineStr"/>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E326" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18299/anthony-medical-centre</t>
@@ -7902,7 +9202,11 @@
           <t>'+971 6 563 0555</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr"/>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E327" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152770/antony-medical-centre</t>
@@ -7925,7 +9229,11 @@
           <t>'+971 6 538 7199</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr"/>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E328" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18301/apollo-medical-clinic</t>
@@ -7948,7 +9256,11 @@
           <t>'+971 6 574 8290</t>
         </is>
       </c>
-      <c r="D329" t="inlineStr"/>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E329" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/232623/baniyas-medical-equipment-trading</t>
@@ -7971,7 +9283,11 @@
           <t>'+971 6 532 8558</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr"/>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E330" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333644/bilal-medical-centre</t>
@@ -7994,7 +9310,11 @@
           <t>'+971 6 562 0181</t>
         </is>
       </c>
-      <c r="D331" t="inlineStr"/>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E331" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153272/chithra-shamsudheens-clinic-dr</t>
@@ -8017,7 +9337,11 @@
           <t>'+971 6 568 5466</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr"/>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E332" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153734/chinese-clinic-the</t>
@@ -8040,7 +9364,11 @@
           <t>'+971 6 524 3444</t>
         </is>
       </c>
-      <c r="D333" t="inlineStr"/>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E333" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18372/cocoon-individualized-natal-care</t>
@@ -8063,7 +9391,11 @@
           <t>'+971 6 533 5555</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr"/>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E334" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18376/consultant-polymedic</t>
@@ -8086,7 +9418,11 @@
           <t>'+971 6 561 8801</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr"/>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E335" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333736/derma-health</t>
@@ -8109,7 +9445,11 @@
           <t>'+971 6 558 4335</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr"/>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E336" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18408/deva-medical-centre</t>
@@ -8132,7 +9472,11 @@
           <t>'+971 6 562 0181</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr"/>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E337" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18453/dr-chithra-shamsudheens-clinic</t>
@@ -8155,7 +9499,11 @@
           <t>'+971 6 561 6261</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr"/>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E338" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18506/dr-maged-salah-eldin</t>
@@ -8178,7 +9526,11 @@
           <t>'+971 6 573 9899</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr"/>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E339" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18515/dr-mariyam-dental-clinic</t>
@@ -8201,7 +9553,11 @@
           <t>'+971 6 555 2116</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr"/>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E340" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18525/dr-mohd-ahmed-ali-dental-clinic</t>
@@ -8224,7 +9580,11 @@
           <t>'+971 6 556 5568</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr"/>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E341" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18551/dr-rabha-habib-el-sayegh-clinic</t>
@@ -8247,7 +9607,11 @@
           <t>'+971 6 569 0569</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr"/>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E342" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/18558/dr-ravindran-gopal-clinic</t>
@@ -8270,7 +9634,11 @@
           <t>'+971 6 555 1666</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr"/>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E343" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/152775/emirates-pvt-poly-clinic</t>
@@ -8293,7 +9661,11 @@
           <t>'+971 6 573 6866</t>
         </is>
       </c>
-      <c r="D344" t="inlineStr"/>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E344" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/236644/emirates-medical-lab</t>
@@ -8316,7 +9688,11 @@
           <t>'+971 6 556 3433</t>
         </is>
       </c>
-      <c r="D345" t="inlineStr"/>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E345" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333741/enjab-hospital-for-day-care</t>
@@ -8339,7 +9715,11 @@
           <t>'+971 6 556 0002</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr"/>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E346" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153409/ent-specialized-clinic</t>
@@ -8362,7 +9742,11 @@
           <t>'+971 6 559 1110</t>
         </is>
       </c>
-      <c r="D347" t="inlineStr"/>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E347" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153112/gayatree-medical-centre</t>
@@ -8385,7 +9769,11 @@
           <t>'+971 6 568 5620</t>
         </is>
       </c>
-      <c r="D348" t="inlineStr"/>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E348" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153117/hayat-medical-centre</t>
@@ -8408,7 +9796,11 @@
           <t>'+971 6 563 5029</t>
         </is>
       </c>
-      <c r="D349" t="inlineStr"/>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E349" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153308/hejazis-clinic-dr</t>
@@ -8431,7 +9823,11 @@
           <t>'+971 6 568 7000</t>
         </is>
       </c>
-      <c r="D350" t="inlineStr"/>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E350" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153438/islamic-medical-herbs-treatment-center</t>
@@ -8454,7 +9850,11 @@
           <t>'+971 6 568 7255</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr"/>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E351" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/240841/ismail-mohd-al-nimir</t>
@@ -8477,7 +9877,11 @@
           <t>'+971 6 572 4855</t>
         </is>
       </c>
-      <c r="D352" t="inlineStr"/>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E352" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153361/jwan-s-murad-clinic-dr</t>
@@ -8500,7 +9904,11 @@
           <t>'+971 6 562 4725</t>
         </is>
       </c>
-      <c r="D353" t="inlineStr"/>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E353" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153249/kottakkal-health-massage</t>
@@ -8523,7 +9931,11 @@
           <t>'+971 6 561 6261</t>
         </is>
       </c>
-      <c r="D354" t="inlineStr"/>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E354" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153746/maged-salah-el-din-clinic-dr</t>
@@ -8546,7 +9958,11 @@
           <t>'+971 6 572 6272</t>
         </is>
       </c>
-      <c r="D355" t="inlineStr"/>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E355" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153371/malek-a-nawas-dr</t>
@@ -8569,7 +9985,11 @@
           <t>'+971 6 572 6272</t>
         </is>
       </c>
-      <c r="D356" t="inlineStr"/>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E356" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153387/malek-abdulla-nawas-dr</t>
@@ -8592,7 +10012,11 @@
           <t>'+971 6 568 5557</t>
         </is>
       </c>
-      <c r="D357" t="inlineStr"/>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E357" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333664/mandar-medical-centre</t>
@@ -8615,7 +10039,11 @@
           <t>'+971 6 573 9899</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr"/>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E358" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153262/mariyam-dental-clinic-dr</t>
@@ -8638,7 +10066,11 @@
           <t>'+971 6 572 2999</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr"/>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E359" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153381/metawi-medical-clinic</t>
@@ -8661,7 +10093,11 @@
           <t>'+971 6 574 9610</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr"/>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E360" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333734/minal-specialised-clinic-dermatology</t>
@@ -8684,7 +10120,11 @@
           <t>'+971 6 555 2116</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr"/>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E361" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153510/mohd-ahamad-ali-dental-clinic-dr</t>
@@ -8707,7 +10147,11 @@
           <t>'+971 6 561 7755</t>
         </is>
       </c>
-      <c r="D362" t="inlineStr"/>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E362" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/153331/mount-seena-medical-centre</t>
@@ -8730,7 +10174,11 @@
           <t>'+971(6)384166</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr"/>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E363" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/299599/nadd-al-shiba-vet-clinic</t>
@@ -8753,7 +10201,11 @@
           <t>'+971 6 534 6522</t>
         </is>
       </c>
-      <c r="D364" t="inlineStr"/>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>kiwavix919@dwseal.co</t>
+        </is>
+      </c>
       <c r="E364" t="inlineStr">
         <is>
           <t>https://www.yello.ae/company/333669/nanda-medical-centre</t>

</xml_diff>